<commit_message>
Update replication package to v1.0.2
</commit_message>
<xml_diff>
--- a/02_Zero_Shot/outputs/Embedding/ALBERT-base-v2/RESULT_clap_albert-base-v2_zeroshot.xlsx
+++ b/02_Zero_Shot/outputs/Embedding/ALBERT-base-v2/RESULT_clap_albert-base-v2_zeroshot.xlsx
@@ -51529,7 +51529,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6.745737925999947</v>
+        <v>30.45318972699897</v>
       </c>
     </row>
     <row r="8">
@@ -51539,7 +51539,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.002248579308666649</v>
+        <v>0.01015106324233299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>